<commit_message>
Small changes. Nothing too major. It was to the spin fluctuation code
</commit_message>
<xml_diff>
--- a/Data/Data comparison - sina and koki temp fluc.xlsx
+++ b/Data/Data comparison - sina and koki temp fluc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cfeb45fc6e4a9cc1/Desktop/Grad school stuff/Research_Notes/Kolodrubetz Group/Cavity QED/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cfeb45fc6e4a9cc1/Desktop/Grad school stuff/Research_Notes/Kolodrubetz Group/Cavity QED/Open_Cavity_QED/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="244" documentId="11_F25DC773A252ABDACC1048D0F11E53185ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3A8CF35-FFA3-4D6C-9114-FD27E60759F9}"/>
+  <xr:revisionPtr revIDLastSave="246" documentId="11_F25DC773A252ABDACC1048D0F11E53185ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8B40934-4254-449A-A7B5-971182D15D4D}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1317,16 +1317,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>628649</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>142874</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61912</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>685797</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>119060</xdr:rowOff>
+      <xdr:colOff>871537</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>109538</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1352,10 +1352,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1826,23 +1822,23 @@
         <v>0.1</v>
       </c>
       <c r="I15">
-        <f xml:space="preserve"> ABS(B14 - B34)</f>
+        <f t="shared" ref="I15:I21" si="0" xml:space="preserve"> ABS(B14 - B34)</f>
         <v>3.9084013803147855E-12</v>
       </c>
       <c r="J15">
-        <f t="shared" ref="J15:J21" si="0" xml:space="preserve"> ABS(C14 - C34)</f>
+        <f t="shared" ref="J15:J21" si="1" xml:space="preserve"> ABS(C14 - C34)</f>
         <v>1.2915992060602566E-14</v>
       </c>
       <c r="K15">
-        <f t="shared" ref="K15:K21" si="1" xml:space="preserve"> ABS(D14 - D34)</f>
+        <f t="shared" ref="K15:K21" si="2" xml:space="preserve"> ABS(D14 - D34)</f>
         <v>1.866940005368356E-10</v>
       </c>
       <c r="L15">
-        <f t="shared" ref="L15:L21" si="2" xml:space="preserve"> ABS(E14 - E34)</f>
+        <f t="shared" ref="L15:L21" si="3" xml:space="preserve"> ABS(E14 - E34)</f>
         <v>1.8000011203778143E-13</v>
       </c>
       <c r="M15">
-        <f t="shared" ref="M15:M21" si="3" xml:space="preserve"> ABS(F14 - F34)</f>
+        <f t="shared" ref="M15:M20" si="4" xml:space="preserve"> ABS(F14 - F34)</f>
         <v>1.5610082670924896E-13</v>
       </c>
     </row>
@@ -1871,23 +1867,23 @@
         <v>0.15</v>
       </c>
       <c r="I16">
-        <f xml:space="preserve"> ABS(B15 - B35)</f>
+        <f t="shared" si="0"/>
         <v>1.5583798140816896E-11</v>
       </c>
       <c r="J16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.4119974680741896E-15</v>
       </c>
       <c r="K16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.0002300083497033E-11</v>
       </c>
       <c r="L16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.6279928474274357E-13</v>
       </c>
       <c r="M16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.892999645924931E-13</v>
       </c>
     </row>
@@ -1916,23 +1912,23 @@
         <v>0.2</v>
       </c>
       <c r="I17">
-        <f xml:space="preserve"> ABS(B16 - B36)</f>
+        <f t="shared" si="0"/>
         <v>8.3982994170117564E-12</v>
       </c>
       <c r="J17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.3929968250013811E-15</v>
       </c>
       <c r="K17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.4043961266428937E-12</v>
       </c>
       <c r="L17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.5000088644850962E-14</v>
       </c>
       <c r="M17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>4.0262931877421693E-13</v>
       </c>
     </row>
@@ -1961,23 +1957,23 @@
         <v>0.25</v>
       </c>
       <c r="I18">
-        <f xml:space="preserve"> ABS(B17 - B37)</f>
+        <f t="shared" si="0"/>
         <v>3.6682802628806854E-11</v>
       </c>
       <c r="J18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.4219879294421549E-15</v>
       </c>
       <c r="K18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.6925198182148335E-11</v>
       </c>
       <c r="L18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.0848999610079133E-12</v>
       </c>
       <c r="M18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.660008935866486E-13</v>
       </c>
     </row>
@@ -2006,23 +2002,23 @@
         <v>0.3</v>
       </c>
       <c r="I19">
-        <f xml:space="preserve"> ABS(B18 - B38)</f>
+        <f t="shared" si="0"/>
         <v>1.7755259935914314E-11</v>
       </c>
       <c r="J19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.6860024621155887E-15</v>
       </c>
       <c r="K19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5597995945148E-12</v>
       </c>
       <c r="L19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.6089881083611886E-13</v>
       </c>
       <c r="M19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5.7470000980330838E-13</v>
       </c>
     </row>
@@ -2048,23 +2044,23 @@
         <v>0.35</v>
       </c>
       <c r="I20">
-        <f xml:space="preserve"> ABS(B19 - B39)</f>
+        <f t="shared" si="0"/>
         <v>8.145300406381395E-12</v>
       </c>
       <c r="J20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.4405390902648705E-16</v>
       </c>
       <c r="K20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.3316099878888394E-11</v>
       </c>
       <c r="L20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0294994023940518E-12</v>
       </c>
       <c r="M20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.8521976447315467E-13</v>
       </c>
     </row>
@@ -2074,19 +2070,19 @@
         <v>0.4</v>
       </c>
       <c r="I21">
-        <f xml:space="preserve"> ABS(B20 - B40)</f>
+        <f t="shared" si="0"/>
         <v>1.6323900564607641E-11</v>
       </c>
       <c r="J21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.6500221088404707E-15</v>
       </c>
       <c r="K21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.2270913132352916E-12</v>
       </c>
       <c r="L21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.5172698087393428E-12</v>
       </c>
     </row>

</xml_diff>